<commit_message>
Fix corrupted Excel files (reconstruits proprement avec openpyxl)
Les fichiers reseau-catemarketing-3nnl.xlsx et reseau-yugo-jnts.xlsx
etaient corrompus a la source (zip invalide, CRC errones). Reconstruits
depuis le classeur regie_tarification_finale.xlsx (RECHERCHE_LYCEES /
RECHERCHE_CAMPUS) avec openpyxl, verifies sains (unzip -t) avant commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEyurFSL9yBPyaLqZBWFM1
</commit_message>
<xml_diff>
--- a/reseau-catemarketing-3nnl.xlsx
+++ b/reseau-catemarketing-3nnl.xlsx
@@ -1,3 +1,18 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Réseau" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
@@ -390,4 +405,1026 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Région</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Département</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ville</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>École</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Typologie d'étude</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Discipline / Filière</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Zone attribuée</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alpes-Maritimes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Alpes-Maritimes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Lycée Régional Hôtelier Jeanne Et Paul Augier</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Polyvalent (sthr - Bac pro cuisine - Service - Boulangerie - Bts)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Calvados</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Caen</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Camille Claudel</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CAEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bourgogne-Franche-Comté</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Côte-D'Or</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dijon</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Lycée Le Castel (Section Hôtelière)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Techno - Bac pro cuisine - Service - Boulangerie - Pâtisserie)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>DIJON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Eure</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Louviers</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Jean-Baptiste Decrétot</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine - Alimentation et boulangerie)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EVREUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Finistère</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Quimperlé</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Roz Glas</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine - Alimentation - Commerce</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>QUIMPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nouvelle-Aquitaine</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gironde</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Talence</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Lycée Hôtelier De Guyenne</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Cuisine - Tourisme) - Cap - Bac pro - Sthr</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>BORDEAUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Grand Est</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Haut-Rhin</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ribeauvillé</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Ribeauvillé (Lycée Du Haut-Rhin)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>COLMAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Occitanie</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Haute-Garonne</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Renée Bonnet</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine - Alimentation)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TOULOUSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hauts-De-Seine</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Clichy</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Lycée Polyvalent René Auffray</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Général</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Polyvalent - Cuisine</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ÎLE-DE-FRANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ille-Et-Vilaine</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Louis Guilloux</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Pro - Boulangerie - Pâtisserie - Cuisine - Soins)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Centre-Val de Loire</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Indre-Et-Loire</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tours</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Lycée Privé Notre-Dame La Riche</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Général - Techno - Pro - Cuisine - Santé - Social)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>TOURS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Centre-Val de Loire</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Indre-Et-Loire</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Amboise</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Lycée Privé Saint-Denis (Antenne)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Général</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Général - Section européenne hôtelière rattachée - Cadre d'ouverture internationale</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>TOURS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Centre-Val de Loire</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Loir-Et-Cher</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Blois</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Lycée Hôtelier Et De Tourisme Du Val De Loire</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Polyvalent national (sthr - Bac pro cuisine - Service - Boulangerie - Pâtisserie - Tourisme d'excellence)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>BLOIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pays de la Loire</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Loire-Atlantique</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Le Pouliguen</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Privé Kerouanaise</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine - Cuisine de terroir et service)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>SAINT-NAZAIRE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pays de la Loire</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Maine-Et-Loire</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Saumur</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Sadi Carnot - Jean Bertin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine - Horlogerie d'art et de précision)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ANGERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Privé Des Métiers De L'Hôtellerie Jean Drouant</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ÎLE-DE-FRANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel École Des Métiers De La Table</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ÎLE-DE-FRANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Privé Charles De Gaulle</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ÎLE-DE-FRANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Nouvelle-Aquitaine</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pyrénées-Atlantiques</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Biarritz</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Lycée Hôtelier De Biarritz</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Cuisine - Sthr - Bac pro cuisine - Service)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>BAYONNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Occitanie</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pyrénées-Orientales</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Canet-En-Roussillon</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Lycée Professionnel Rosa Luxembourg</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Pro - Cuisine - Tourisme et services de proximité)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>PERPIGNAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Auvergne-Rhône-Alpes</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Savoie</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Aix-Les-Bains / Chambéry Couronne</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Lycée Marlioz (Bassin Élargi)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Techno</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Général - Techno - Cuisine</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>CHAMBERY</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Auvergne-Rhône-Alpes</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Savoie</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Bourg-Saint-Maurice</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Lycée Saint-Exupéry</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Général - Pro - Cuisine</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>CHAMBERY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Nouvelle-Aquitaine</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Vienne</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Poitiers / Grand Poitiers</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Lycée Des Métiers De L'Hôtellerie Et Du Tourisme (Lycée Aliénor D'Aquitaine)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Lycée</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Techno</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Techno - Cuisine - Tourisme)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>POITIERS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>